<commit_message>
auto: 更新 HK Swing 2026-07-25
</commit_message>
<xml_diff>
--- a/hk_swing_pattern/HK_Swing_Pattern.xlsx
+++ b/hk_swing_pattern/HK_Swing_Pattern.xlsx
@@ -3405,7 +3405,9 @@
       <c r="I46" s="2" t="inlineStr"/>
       <c r="J46" s="2" t="inlineStr"/>
       <c r="K46" s="2" t="inlineStr"/>
-      <c r="L46" s="2" t="inlineStr"/>
+      <c r="L46" s="2" t="n">
+        <v>9</v>
+      </c>
       <c r="M46" s="2" t="inlineStr"/>
       <c r="N46" s="2" t="n">
         <v>4</v>
@@ -5400,7 +5402,9 @@
       <c r="J78" s="2" t="inlineStr"/>
       <c r="K78" s="2" t="inlineStr"/>
       <c r="L78" s="2" t="inlineStr"/>
-      <c r="M78" s="2" t="inlineStr"/>
+      <c r="M78" s="2" t="n">
+        <v>9</v>
+      </c>
       <c r="N78" s="2" t="n">
         <v>0</v>
       </c>
@@ -11897,7 +11901,9 @@
       <c r="I184" s="2" t="inlineStr"/>
       <c r="J184" s="2" t="inlineStr"/>
       <c r="K184" s="2" t="inlineStr"/>
-      <c r="L184" s="2" t="inlineStr"/>
+      <c r="L184" s="2" t="n">
+        <v>9</v>
+      </c>
       <c r="M184" s="2" t="inlineStr"/>
       <c r="N184" s="2" t="n">
         <v>0</v>
@@ -13259,7 +13265,9 @@
       <c r="I206" s="2" t="inlineStr"/>
       <c r="J206" s="2" t="inlineStr"/>
       <c r="K206" s="2" t="inlineStr"/>
-      <c r="L206" s="2" t="inlineStr"/>
+      <c r="L206" s="2" t="n">
+        <v>9</v>
+      </c>
       <c r="M206" s="2" t="n">
         <v>9</v>
       </c>
@@ -14293,7 +14301,9 @@
         <v>1</v>
       </c>
       <c r="K223" s="2" t="inlineStr"/>
-      <c r="L223" s="2" t="inlineStr"/>
+      <c r="L223" s="2" t="n">
+        <v>9</v>
+      </c>
       <c r="M223" s="2" t="n">
         <v>9</v>
       </c>
@@ -15076,7 +15086,9 @@
       <c r="L236" s="2" t="n">
         <v>9</v>
       </c>
-      <c r="M236" s="2" t="inlineStr"/>
+      <c r="M236" s="2" t="n">
+        <v>-9</v>
+      </c>
       <c r="N236" s="2" t="n">
         <v>0</v>
       </c>
@@ -15246,7 +15258,9 @@
       <c r="J239" s="2" t="inlineStr"/>
       <c r="K239" s="2" t="inlineStr"/>
       <c r="L239" s="2" t="inlineStr"/>
-      <c r="M239" s="2" t="inlineStr"/>
+      <c r="M239" s="2" t="n">
+        <v>9</v>
+      </c>
       <c r="N239" s="2" t="n">
         <v>1</v>
       </c>
@@ -16701,7 +16715,9 @@
       <c r="I264" s="2" t="inlineStr"/>
       <c r="J264" s="2" t="inlineStr"/>
       <c r="K264" s="2" t="inlineStr"/>
-      <c r="L264" s="2" t="inlineStr"/>
+      <c r="L264" s="2" t="n">
+        <v>-9</v>
+      </c>
       <c r="M264" s="2" t="n">
         <v>-13</v>
       </c>
@@ -17050,7 +17066,9 @@
       <c r="J270" s="2" t="inlineStr"/>
       <c r="K270" s="2" t="inlineStr"/>
       <c r="L270" s="2" t="inlineStr"/>
-      <c r="M270" s="2" t="inlineStr"/>
+      <c r="M270" s="2" t="n">
+        <v>-9</v>
+      </c>
       <c r="N270" s="2" t="n">
         <v>0</v>
       </c>
@@ -17296,7 +17314,9 @@
       </c>
       <c r="K274" s="2" t="inlineStr"/>
       <c r="L274" s="2" t="inlineStr"/>
-      <c r="M274" s="2" t="inlineStr"/>
+      <c r="M274" s="2" t="n">
+        <v>-9</v>
+      </c>
       <c r="N274" s="2" t="n">
         <v>2</v>
       </c>
@@ -18287,7 +18307,9 @@
       <c r="I291" s="2" t="inlineStr"/>
       <c r="J291" s="2" t="inlineStr"/>
       <c r="K291" s="2" t="inlineStr"/>
-      <c r="L291" s="2" t="inlineStr"/>
+      <c r="L291" s="2" t="n">
+        <v>9</v>
+      </c>
       <c r="M291" s="2" t="inlineStr"/>
       <c r="N291" s="2" t="n">
         <v>0</v>
@@ -19737,7 +19759,9 @@
       <c r="I315" s="2" t="inlineStr"/>
       <c r="J315" s="2" t="inlineStr"/>
       <c r="K315" s="2" t="inlineStr"/>
-      <c r="L315" s="2" t="inlineStr"/>
+      <c r="L315" s="2" t="n">
+        <v>9</v>
+      </c>
       <c r="M315" s="2" t="inlineStr"/>
       <c r="N315" s="2" t="n">
         <v>0</v>
@@ -23117,7 +23141,9 @@
       <c r="I371" s="2" t="inlineStr"/>
       <c r="J371" s="2" t="inlineStr"/>
       <c r="K371" s="2" t="inlineStr"/>
-      <c r="L371" s="2" t="inlineStr"/>
+      <c r="L371" s="2" t="n">
+        <v>9</v>
+      </c>
       <c r="M371" s="2" t="inlineStr"/>
       <c r="N371" s="2" t="n">
         <v>1</v>
@@ -26853,7 +26879,9 @@
       <c r="I433" s="2" t="inlineStr"/>
       <c r="J433" s="2" t="inlineStr"/>
       <c r="K433" s="2" t="inlineStr"/>
-      <c r="L433" s="2" t="inlineStr"/>
+      <c r="L433" s="2" t="n">
+        <v>9</v>
+      </c>
       <c r="M433" s="2" t="n">
         <v>9</v>
       </c>
@@ -27245,7 +27273,9 @@
         <v>1</v>
       </c>
       <c r="K439" s="2" t="inlineStr"/>
-      <c r="L439" s="2" t="inlineStr"/>
+      <c r="L439" s="2" t="n">
+        <v>9</v>
+      </c>
       <c r="M439" s="2" t="inlineStr"/>
       <c r="N439" s="2" t="n">
         <v>0</v>
@@ -28715,7 +28745,9 @@
       <c r="I463" s="2" t="inlineStr"/>
       <c r="J463" s="2" t="inlineStr"/>
       <c r="K463" s="2" t="inlineStr"/>
-      <c r="L463" s="2" t="inlineStr"/>
+      <c r="L463" s="2" t="n">
+        <v>-9</v>
+      </c>
       <c r="M463" s="2" t="inlineStr"/>
       <c r="N463" s="2" t="n">
         <v>2</v>

</xml_diff>

<commit_message>
auto: 更新 HK Swing 2026-07-29
</commit_message>
<xml_diff>
--- a/hk_swing_pattern/HK_Swing_Pattern.xlsx
+++ b/hk_swing_pattern/HK_Swing_Pattern.xlsx
@@ -5124,7 +5124,9 @@
         <v>1</v>
       </c>
       <c r="P72" s="2" t="inlineStr"/>
-      <c r="Q72" s="2" t="inlineStr"/>
+      <c r="Q72" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="R72" s="2" t="inlineStr"/>
       <c r="S72" s="2" t="inlineStr"/>
       <c r="T72" s="2" t="inlineStr"/>
@@ -5248,7 +5250,9 @@
       </c>
       <c r="O74" s="2" t="inlineStr"/>
       <c r="P74" s="2" t="inlineStr"/>
-      <c r="Q74" s="2" t="inlineStr"/>
+      <c r="Q74" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="R74" s="2" t="inlineStr"/>
       <c r="S74" s="2" t="inlineStr"/>
       <c r="T74" s="2" t="inlineStr"/>
@@ -11224,7 +11228,9 @@
       </c>
       <c r="O169" s="2" t="inlineStr"/>
       <c r="P169" s="2" t="inlineStr"/>
-      <c r="Q169" s="2" t="inlineStr"/>
+      <c r="Q169" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="R169" s="2" t="inlineStr"/>
       <c r="S169" s="2" t="inlineStr"/>
       <c r="T169" s="2" t="inlineStr"/>
@@ -11552,7 +11558,9 @@
       <c r="P174" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="Q174" s="2" t="inlineStr"/>
+      <c r="Q174" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="R174" s="2" t="inlineStr"/>
       <c r="S174" s="2" t="inlineStr"/>
       <c r="T174" s="2" t="inlineStr"/>
@@ -11936,7 +11944,9 @@
         <v>1</v>
       </c>
       <c r="P180" s="2" t="inlineStr"/>
-      <c r="Q180" s="2" t="inlineStr"/>
+      <c r="Q180" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="R180" s="2" t="n">
         <v>-1</v>
       </c>
@@ -12130,7 +12140,9 @@
       <c r="P183" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="Q183" s="2" t="inlineStr"/>
+      <c r="Q183" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="R183" s="2" t="inlineStr">
         <is>
           <t>预-1</t>
@@ -15586,7 +15598,9 @@
       <c r="P240" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="Q240" s="2" t="inlineStr"/>
+      <c r="Q240" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="R240" s="2" t="n">
         <v>1</v>
       </c>
@@ -21036,7 +21050,9 @@
       </c>
       <c r="O328" s="2" t="inlineStr"/>
       <c r="P328" s="2" t="inlineStr"/>
-      <c r="Q328" s="2" t="inlineStr"/>
+      <c r="Q328" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="R328" s="2" t="n">
         <v>1</v>
       </c>
@@ -25356,7 +25372,9 @@
       </c>
       <c r="O398" s="2" t="inlineStr"/>
       <c r="P398" s="2" t="inlineStr"/>
-      <c r="Q398" s="2" t="inlineStr"/>
+      <c r="Q398" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="R398" s="2" t="n">
         <v>1</v>
       </c>
@@ -27826,7 +27844,9 @@
       </c>
       <c r="O437" s="2" t="inlineStr"/>
       <c r="P437" s="2" t="inlineStr"/>
-      <c r="Q437" s="2" t="inlineStr"/>
+      <c r="Q437" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="R437" s="2" t="n">
         <v>-1</v>
       </c>
@@ -29194,9 +29214,7 @@
         <v>1</v>
       </c>
       <c r="P459" s="2" t="inlineStr"/>
-      <c r="Q459" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="Q459" s="2" t="inlineStr"/>
       <c r="R459" s="2" t="n">
         <v>1</v>
       </c>
@@ -29376,7 +29394,9 @@
       </c>
       <c r="O462" s="2" t="inlineStr"/>
       <c r="P462" s="2" t="inlineStr"/>
-      <c r="Q462" s="2" t="inlineStr"/>
+      <c r="Q462" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="R462" s="2" t="inlineStr"/>
       <c r="S462" s="2" t="inlineStr"/>
       <c r="T462" s="2" t="n">
@@ -29688,7 +29708,9 @@
       </c>
       <c r="O467" s="2" t="inlineStr"/>
       <c r="P467" s="2" t="inlineStr"/>
-      <c r="Q467" s="2" t="inlineStr"/>
+      <c r="Q467" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="R467" s="2" t="inlineStr"/>
       <c r="S467" s="2" t="inlineStr"/>
       <c r="T467" s="2" t="inlineStr"/>

</xml_diff>

<commit_message>
auto: 更新 HK Swing 2026-08-09
</commit_message>
<xml_diff>
--- a/hk_swing_pattern/HK_Swing_Pattern.xlsx
+++ b/hk_swing_pattern/HK_Swing_Pattern.xlsx
@@ -22264,25 +22264,25 @@
       <c r="T349" s="2" t="inlineStr"/>
       <c r="U349" s="2" t="inlineStr"/>
       <c r="V349" s="2" t="n">
-        <v>-80.27</v>
+        <v>-81.65000000000001</v>
       </c>
       <c r="W349" s="2" t="n">
-        <v>-50.77</v>
+        <v>-50.72</v>
       </c>
       <c r="X349" s="2" t="n">
         <v>2.46</v>
       </c>
       <c r="Y349" s="2" t="n">
-        <v>-15.21</v>
+        <v>-15.22</v>
       </c>
       <c r="Z349" s="2" t="n">
-        <v>-50.52</v>
+        <v>-50.44</v>
       </c>
       <c r="AA349" s="2" t="n">
-        <v>3.35</v>
+        <v>3.36</v>
       </c>
       <c r="AB349" s="2" t="n">
-        <v>-13.82</v>
+        <v>-13.84</v>
       </c>
     </row>
     <row r="350">

</xml_diff>

<commit_message>
auto: 更新 HK Swing 2026-08-15
</commit_message>
<xml_diff>
--- a/hk_swing_pattern/HK_Swing_Pattern.xlsx
+++ b/hk_swing_pattern/HK_Swing_Pattern.xlsx
@@ -28814,25 +28814,25 @@
       <c r="T457" s="2" t="inlineStr"/>
       <c r="U457" s="2" t="inlineStr"/>
       <c r="V457" s="2" t="n">
-        <v>-62.8</v>
+        <v>-62.71</v>
       </c>
       <c r="W457" s="2" t="n">
-        <v>-30.91</v>
+        <v>-30.54</v>
       </c>
       <c r="X457" s="2" t="n">
-        <v>-3.07</v>
+        <v>-2.7</v>
       </c>
       <c r="Y457" s="2" t="n">
-        <v>13.27</v>
+        <v>13.64</v>
       </c>
       <c r="Z457" s="2" t="n">
-        <v>-32.02</v>
+        <v>-31.66</v>
       </c>
       <c r="AA457" s="2" t="n">
-        <v>-4.51</v>
+        <v>-4.15</v>
       </c>
       <c r="AB457" s="2" t="n">
-        <v>13.73</v>
+        <v>14.1</v>
       </c>
     </row>
     <row r="458">

</xml_diff>

<commit_message>
auto: 更新 HK Swing 2026-08-17
</commit_message>
<xml_diff>
--- a/hk_swing_pattern/HK_Swing_Pattern.xlsx
+++ b/hk_swing_pattern/HK_Swing_Pattern.xlsx
@@ -579,12 +579,12 @@
       </c>
       <c r="P1" s="1" t="inlineStr">
         <is>
-          <t>SOS_orig</t>
+          <t>SOS</t>
         </is>
       </c>
       <c r="Q1" s="1" t="inlineStr">
         <is>
-          <t>SOS</t>
+          <t>SOS_过去3日</t>
         </is>
       </c>
       <c r="R1" s="1" t="inlineStr">
@@ -971,9 +971,7 @@
         <v>0</v>
       </c>
       <c r="O7" s="2" t="inlineStr"/>
-      <c r="P7" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="P7" s="2" t="inlineStr"/>
       <c r="Q7" s="2" t="n">
         <v>1</v>
       </c>
@@ -3318,7 +3316,9 @@
       </c>
       <c r="O44" s="2" t="inlineStr"/>
       <c r="P44" s="2" t="inlineStr"/>
-      <c r="Q44" s="2" t="inlineStr"/>
+      <c r="Q44" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="R44" s="2" t="n">
         <v>-1</v>
       </c>
@@ -7751,9 +7751,7 @@
         <v>0</v>
       </c>
       <c r="O115" s="2" t="inlineStr"/>
-      <c r="P115" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="P115" s="2" t="inlineStr"/>
       <c r="Q115" s="2" t="n">
         <v>1</v>
       </c>
@@ -8143,9 +8141,7 @@
         <v>1</v>
       </c>
       <c r="O121" s="2" t="inlineStr"/>
-      <c r="P121" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="P121" s="2" t="inlineStr"/>
       <c r="Q121" s="2" t="n">
         <v>1</v>
       </c>
@@ -9825,9 +9821,7 @@
         <v>0</v>
       </c>
       <c r="O148" s="2" t="inlineStr"/>
-      <c r="P148" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="P148" s="2" t="inlineStr"/>
       <c r="Q148" s="2" t="n">
         <v>1</v>
       </c>
@@ -10536,7 +10530,9 @@
         <v>1</v>
       </c>
       <c r="P159" s="2" t="inlineStr"/>
-      <c r="Q159" s="2" t="inlineStr"/>
+      <c r="Q159" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="R159" s="2" t="inlineStr">
         <is>
           <t>预-1</t>
@@ -13299,9 +13295,7 @@
         <v>1</v>
       </c>
       <c r="O203" s="2" t="inlineStr"/>
-      <c r="P203" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="P203" s="2" t="inlineStr"/>
       <c r="Q203" s="2" t="n">
         <v>1</v>
       </c>
@@ -16244,7 +16238,9 @@
         <v>1</v>
       </c>
       <c r="P252" s="2" t="inlineStr"/>
-      <c r="Q252" s="2" t="inlineStr"/>
+      <c r="Q252" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="R252" s="2" t="inlineStr">
         <is>
           <t>预-1</t>
@@ -18529,9 +18525,7 @@
         <v>0</v>
       </c>
       <c r="O290" s="2" t="inlineStr"/>
-      <c r="P290" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="P290" s="2" t="inlineStr"/>
       <c r="Q290" s="2" t="n">
         <v>1</v>
       </c>
@@ -20113,9 +20107,7 @@
         <v>0</v>
       </c>
       <c r="O315" s="2" t="inlineStr"/>
-      <c r="P315" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="P315" s="2" t="inlineStr"/>
       <c r="Q315" s="2" t="n">
         <v>1</v>
       </c>
@@ -22865,9 +22857,7 @@
         <v>0</v>
       </c>
       <c r="O360" s="2" t="inlineStr"/>
-      <c r="P360" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="P360" s="2" t="inlineStr"/>
       <c r="Q360" s="2" t="n">
         <v>1</v>
       </c>
@@ -23050,7 +23040,7 @@
         </is>
       </c>
       <c r="T363" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="U363" s="2" t="inlineStr"/>
       <c r="V363" s="2" t="n">
@@ -23412,9 +23402,7 @@
       <c r="P369" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="Q369" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="Q369" s="2" t="inlineStr"/>
       <c r="R369" s="2" t="n">
         <v>1</v>
       </c>
@@ -25347,9 +25335,7 @@
         <v>0</v>
       </c>
       <c r="O400" s="2" t="inlineStr"/>
-      <c r="P400" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="P400" s="2" t="inlineStr"/>
       <c r="Q400" s="2" t="n">
         <v>1</v>
       </c>
@@ -27851,10 +27837,10 @@
         <v>0</v>
       </c>
       <c r="O441" s="2" t="inlineStr"/>
-      <c r="P441" s="2" t="inlineStr"/>
-      <c r="Q441" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="P441" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q441" s="2" t="inlineStr"/>
       <c r="R441" s="2" t="n">
         <v>1</v>
       </c>
@@ -32407,7 +32393,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A41"/>
+  <dimension ref="A1:A43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -32547,130 +32533,144 @@
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">  SOS_orig (原版 SoS): 近3日, 60日区间pos&lt;=0.50 + 放量&gt;=1.5x + 阳线(body&gt;=3%&amp;range&gt;=1.5x&amp;close_pos&gt;=0.70)。纯底部反强, 无均线纠缠</t>
+          <t xml:space="preserve">  SOS (Sign of Strength, Wyckoff): 仅看今日最新一根bar。位置门 A OR B, 强度共享放量</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">  SOS (新版 SoS): 位置门 = A OR B。A: 6个月pos&lt;=0.50(6月数据不足回退3个月); B: 近3日 4均线(5/10/15/20)纠缠 max/min-1&lt;5%。强度同原版(放量+阳线)。捕获2328式纠缠平台突破、9980式次新股底部反强</t>
+          <t xml:space="preserve">    位置门A: 200日分位&lt;=0.80(200日不足回退3个月); 位置门B: 近3日 4均线(5/10/15/20)纠缠 max/min-1&lt;5%(平台启动)</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
         <is>
+          <t xml:space="preserve">    强度: 放量&gt;=1.5x + 中大阳(实体&gt;3%) + 波幅扩张(1.5x) + 收盘靠高(&gt;=70%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  SOS_过去3日: 过去3个交易日(不含今日)出现过SOS的个股。用于观察SOS后的股价反应(如缩量回踩不破前低=买点)</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
           <t xml:space="preserve">    阳线path: 中大阳(实体&gt;3%) + 波幅扩张(1.5x) + 收盘靠高(&gt;=70%) + 放量。无十字星路径(小实体不再触发)</t>
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="5" t="inlineStr"/>
-    </row>
-    <row r="26">
-      <c r="A26" s="6" t="inlineStr">
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="6" t="inlineStr">
         <is>
           <t>【④ 企稳上行 — Cross】</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  KDJ Cross / 日MACD Cross / 10_50 Cross: 日线快线上穿慢线=金叉, 下穿=死叉</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    近2日金叉=1 / 死叉=-1; 按gap斜率线性推算将交叉=预1 / 预-1; 否则空</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">    KDJ: K上穿D; MACD: DIF上穿DEA; 10_50: MA10上穿MA50(需close&gt;=MA50)</t>
+          <t xml:space="preserve">  KDJ Cross / 日MACD Cross / 10_50 Cross: 日线快线上穿慢线=金叉, 下穿=死叉</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">    MACD 专属: 预告窗口=3日(其他2日), 且需过去3根MACD柱(DIF-DEA)依次单边且加速, 来回震荡不触发预告</t>
+          <t xml:space="preserve">    近2日金叉=1 / 死叉=-1; 按gap斜率线性推算将交叉=预1 / 预-1; 否则空</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">  5_10 Cross (稳定穿过版, 不报预告): MA5 vs MA10</t>
+          <t xml:space="preserve">    KDJ: K上穿D; MACD: DIF上穿DEA; 10_50: MA10上穿MA50(需close&gt;=MA50)</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">    稳定穿过: gap近2日内过零 且 过零前5日|gap|持续收窄(允许1次反复) → 1金叉/-1死叉</t>
+          <t xml:space="preserve">    MACD 专属: 预告窗口=3日(其他2日), 且需过去3根MACD柱(DIF-DEA)依次单边且加速, 来回震荡不触发预告</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="5" t="inlineStr">
         <is>
+          <t xml:space="preserve">  5_10 Cross (稳定穿过版, 不报预告): MA5 vs MA10</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    稳定穿过: gap近2日内过零 且 过零前5日|gap|持续收窄(允许1次反复) → 1金叉/-1死叉</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
           <t xml:space="preserve">    有过零但不稳定(whipsaw/暴涨驱动等脏交叉) → 0; 无过零但两线持续重叠(近5日rel&lt;0.2%) → 0; 其余空</t>
         </is>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" s="5" t="inlineStr"/>
-    </row>
-    <row r="35">
-      <c r="A35" s="6" t="inlineStr">
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="6" t="inlineStr">
         <is>
           <t>【⑤ HK 专属 — 趋势/Mansfield RS】</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  年线斜率: MA200 近5日变化率 ×52 (年化, %)。正值=年线上行</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  MRS_HSI: Mansfield RS vs 2800.HK(盈富基金,HSI代理) = (个股/2800.HK)/(252日均线)-1 ×100。0=在均线上, 正=跑赢, 负=跑输</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">  MRS_HSI_1W / MRS_HSI_4W: MRS_HSI 分数的 5日 / 20日 变化</t>
+          <t xml:space="preserve">  年线斜率: MA200 近5日变化率 ×52 (年化, %)。正值=年线上行</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">  MRS_HD: Mansfield RS vs 3110.HK(恒生高股息率ETF) = (个股/3110.HK)/(252日均线)-1 ×100。正=跑赢高股息指数</t>
+          <t xml:space="preserve">  MRS_HSI: Mansfield RS vs 2800.HK(盈富基金,HSI代理) = (个股/2800.HK)/(252日均线)-1 ×100。0=在均线上, 正=跑赢, 负=跑输</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">  MRS_HD_1W / MRS_HD_4W: MRS_HD 分数的 5日 / 20日 变化</t>
+          <t xml:space="preserve">  MRS_HSI_1W / MRS_HSI_4W: MRS_HSI 分数的 5日 / 20日 变化</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  MRS_HD: Mansfield RS vs 3110.HK(恒生高股息率ETF) = (个股/3110.HK)/(252日均线)-1 ×100。正=跑赢高股息指数</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  MRS_HD_1W / MRS_HD_4W: MRS_HD 分数的 5日 / 20日 变化</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">  (HK股票池无sector, 不算 MRS_行业)</t>
         </is>

</xml_diff>